<commit_message>
feat(F-NAR-019): ATOM-EMO.GES.002-08 Le pont de Nina
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.GES.002-08.xlsx
+++ b/stories/arbres/ATOM-EMO.GES.002-08.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>salon puis cuisine</t>
+          <t>salon puis cuisine, tabouret, cubes, voiture, soupe, pain, bois, casserole, sol</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nina veut un pont de cubes. Il tombe. Elle souffle, fait une pause. Plus tard, dans la cuisine, elle recommence.</t>
+          <t>La petite voiture tape le tabouret. Sur le bois, un éclat de tabouret luit. Nina veut un pont, maintenant. Le pont tombe. Poitrine trop vite. Sourire parti. Papa s'accroupit. Elle souffle, pause. Merci vécu. Deuxième ruse : la casserole glisse, bruit fort, le corps repart trop vite. Elle refuse de foncer. Un éclat de tabouret tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Sur le toit, la pluie fait des petits coups. Comme des doigts, tout légers. L'odeur de soupe monte de la cuisine. Elle se mélange à l'air du salon. Un tapis bleu attend les pieds. Une voiture en bois dort près du canapé. La casserole est sur le feu, tout doux. Je coupe le pain. Vous jouez au salon ? Oui. Les cubes sont près du tapis. Je veux un pont, papa. Un pont de cubes. J'écoute depuis la cuisine. La voiture pourra passer, plus tard. En ce moment, Nina est sur le tapis bleu. Elle construit un pont avec des cubes. Les cubes cliquent. Le bois est lisse, un peu froid. Tu poses les piles, puis la planche ? Oui. Un pont pour les voitures. Nina pose une planche. Le pont tremble. Le pont tombe. Nina sent son ventre serré. Sa poitrine va trop vite. C'est trop. Je suis fâchée. Le pont est tombé. Tu es fâchée. On souffle. Nina souffle. Un grand souffle. On fait une pause. Nina s'assoit. Elle pose les mains sur ses genoux. Elle souffle encore. La pause est calme. Son ventre se desserre. La pluie continue sur le toit. Je souffle. Je fais une pause. Tu as soufflé. Tu as fait une pause. Bravo, Nina. J'ai entendu. C'est calme. Tu veux reprendre, tout doucement ? Oui. Un petit pont. Nina reprend un cube. Le pont est petit. Il tient.</t>
+          <t>La petite voiture tape le tabouret. Toc, papa. Elle a heurté le bois, Nina ? Oui, le tabouret. Le bois du tabouret sent la soupe, un peu. Ça sent la soupe, maman. Tu la sens, depuis le salon ? Oui, maman. Sur le bois, un éclat de tabouret luit. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Maman coupe le pain, dans la cuisine. Le pain est tiède, sous les doigts. Je le sens d'ici. La casserole chante un peu, Nina. Elle fait un petit bruit. Le salon sent le bois et la soupe, ensemble. Les cubes attendent au sol, lisses et froids. Ils sont froids, papa. Tu les touches, les cubes ? Oui, papa. Nina s'assoit près du tabouret, les genoux pliés. Je veux un pont, maintenant. Un pont pour la voiture ? Oui, tout de suite. En ce moment, Nina prend un cube. Elle veut un pont, très long. La voiture va passer. Tu poses les cubes, Nina ? Oui, papa. Nina pose un cube trop vite. Puis un autre, trop haut. Plus haut ! Le pont penche d'un coup, vers le sol. Les cubes tombent près du tabouret. Ça fait un bruit sec. Oh. Nina reste surprise, les mains ouvertes. Sa poitrine va trop vite. Le sourire de Nina disparaît. C'est trop, papa. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois les cubes, Nina ? Oui, papa. Tes mains sont chaudes, Nina ? Un peu, maman. Un éclat de tabouret tremble, près du sol.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Sur le toit, la pluie fait des petits coups. Comme des doigts, tout légers. L'odeur de soupe monte de la cuisine. Elle se mélange à l'air du salon. Un tapis bleu attend les pieds. Une voiture en bois dort près du canapé. La casserole est sur le feu, tout doux. Je coupe le pain. Vous jouez au salon ? Oui. Les cubes sont près du tapis. Je veux un pont, papa. Un pont de cubes. J'écoute depuis la cuisine. La voiture pourra passer, plus tard. En ce moment, Nina est sur le tapis bleu. Elle construit un pont avec des cubes. Les cubes cliquent. Le bois est lisse, un peu froid. Tu poses les piles, puis la planche ? Oui. Un pont pour les voitures. Nina pose une planche. Le pont tremble. Le pont tombe. Nina sent son ventre serré. Sa poitrine va trop vite. C'est trop. Je suis fâchée. Le pont est tombé. Tu es fâchée. On souffle. Nina souffle. Un grand souffle. On fait une pause. Nina s'assoit. Elle pose les mains sur ses genoux. Elle souffle encore. La pause est calme. Son ventre se desserre. La pluie continue sur le toit. Je souffle. Je fais une pause. Tu as soufflé. Tu as fait une pause. Bravo, Nina. J'ai entendu. C'est calme. Tu veux reprendre, tout doucement ? Oui. Un petit pont. Nina reprend un cube. Le pont est petit. Il tient.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La petite voiture tape le tabouret. Toc, papa. Elle a heurté le bois, Nina ? Oui, le tabouret. Le bois du tabouret sent la soupe, un peu. Ça sent la soupe, maman. Tu la sens, depuis le salon ? Oui, maman. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de tabouret&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Maman coupe le pain, dans la cuisine. Le pain est tiède, sous les doigts. Je le sens d'ici. La casserole chante un peu, Nina. Elle fait un petit bruit. Le salon sent le bois et la soupe, ensemble. Les cubes attendent au sol, lisses et froids. Ils sont froids, papa. Tu les touches, les cubes ? Oui, papa. Nina s'assoit près du tabouret, les genoux pliés. Je veux un pont, maintenant. Un pont pour la voiture ? Oui, tout de suite. En ce moment, Nina prend un cube. Elle veut un pont, très long. La voiture va passer. Tu poses les cubes, Nina ? Oui, papa. Nina pose un cube trop vite. Puis un autre, trop haut. Plus haut ! Le pont penche d'un coup, vers le sol. Les cubes tombent près du tabouret. Ça fait un bruit sec. Oh. Nina reste surprise, les mains ouvertes. Sa poitrine va trop vite. Le sourire de Nina disparaît. C'est trop, papa. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois les cubes, Nina ? Oui, papa. Tes mains sont chaudes, Nina ? Un peu, maman. Un éclat de tabouret tremble, près du sol.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Ferdinand construit un pont avec des cubes. Les cubes cliquent. Le pont tombe. Ferdinand sent son ventre serré. Papa arrive. Papa dit : on souffle. Ferdinand souffle. Un grand souffle. Papa dit : on fait une &lt;emphasis&gt;pause&lt;/emphasis&gt;. Ferdinand s'assoit. Il pose les fesses au tapis. Il souffle encore. La pause est calme. Son ventre se desserre. Plus tard, dans la cuisine, une casserole glisse. Ça fait un bruit fort. Ferdinand sent encore son ventre. Même leçon, autre lieu. Il s'assoit près de maman. Il souffle. Il fait une pause. Puis il reprend. Maman dit : tu as soufflé. Tu as fait une pause. Ferdinand sourit. [pause]</t>
+          <t>La petite voiture tape le tabouret. Toc, papa. Elle a heurté le bois, Nina ? Oui, le tabouret. Le bois du tabouret sent la soupe, un peu. Ça sent la soupe, maman. Tu la sens, depuis le salon ? Oui, maman. Sur le bois, un &lt;emphasis&gt;éclat de tabouret&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Maman coupe le pain, dans la cuisine. Le pain est tiède, sous les doigts. Je le sens d'ici. La casserole chante un peu, Nina. Elle fait un petit bruit. Le salon sent le bois et la soupe, ensemble. Les cubes attendent au sol, lisses et froids. Ils sont froids, papa. Tu les touches, les cubes ? Oui, papa. Nina s'assoit près du tabouret, les genoux pliés. Je veux un pont, maintenant. Un pont pour la voiture ? Oui, tout de suite. En ce moment, Nina prend un cube. Elle veut un pont, très long. La voiture va passer. Tu poses les cubes, Nina ? Oui, papa. Nina pose un cube trop vite. Puis un autre, trop haut. Plus haut ! Le pont penche d'un coup, vers le sol. Les cubes tombent près du tabouret. Ça fait un bruit sec. Oh. Nina reste surprise, les mains ouvertes. Sa poitrine va trop vite. Le sourire de Nina disparaît. C'est trop, papa. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois les cubes, Nina ? Oui, papa. Tes mains sont chaudes, Nina ? Un peu, maman. Un éclat de tabouret tremble, près du sol. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
         <v>1.12</v>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>pause</t>
+          <t>éclat de tabouret</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.96</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,57 +1321,68 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_un_pont_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Sur le toit, la pluie fait des petits coups.
-narrateur|Comme des doigts, tout légers.
-narrateur|L'odeur de soupe monte de la cuisine.
-narrateur|Elle se mélange à l'air du salon.
-narrateur|Un tapis bleu attend les pieds.
-narrateur|Une voiture en bois dort près du canapé.
-papa|La casserole est sur le feu, tout doux.
-maman|Je coupe le pain. Vous jouez au salon ?
-papa|Oui. Les cubes sont près du tapis.
-enfant-f|Je veux un pont, papa.
-maman|Un pont de cubes. J'écoute depuis la cuisine.
-papa|La voiture pourra passer, plus tard.
-narrateur|En ce moment, Nina est sur le tapis bleu.
-narrateur|Elle construit un pont avec des cubes.
-narrateur|Les cubes cliquent.
-narrateur|Le bois est lisse, un peu froid.
-papa|Tu poses les piles, puis la planche ?
-enfant-f|Oui. Un pont pour les voitures.
-narrateur|Nina pose une planche.
-narrateur|Le pont tremble.
-narrateur|Le pont tombe.
-narrateur|Nina sent son ventre serré.
+          <t>narrateur|La petite voiture tape le tabouret.
+enfant-f|Toc, papa.
+papa|Elle a heurté le bois, Nina ?
+enfant-f|Oui, le tabouret.
+narrateur|Le bois du tabouret sent la soupe, un peu.
+enfant-f|Ça sent la soupe, maman.
+maman|Tu la sens, depuis le salon ?
+enfant-f|Oui, maman.
+narrateur|Sur le bois, un éclat de tabouret luit.
+enfant-f|Il brille, papa.
+papa|Tu le vois, le petit point ?
+enfant-f|Oui, un petit point.
+narrateur|Maman coupe le pain, dans la cuisine.
+maman|Le pain est tiède, sous les doigts.
+enfant-f|Je le sens d'ici.
+papa|La casserole chante un peu, Nina.
+enfant-f|Elle fait un petit bruit.
+narrateur|Le salon sent le bois et la soupe, ensemble.
+narrateur|Les cubes attendent au sol, lisses et froids.
+enfant-f|Ils sont froids, papa.
+papa|Tu les touches, les cubes ?
+enfant-f|Oui, papa.
+narrateur|Nina s'assoit près du tabouret, les genoux pliés.
+enfant-f|Je veux un pont, maintenant.
+papa|Un pont pour la voiture ?
+enfant-f|Oui, tout de suite.
+narrateur|En ce moment, Nina prend un cube.
+narrateur|Elle veut un pont, très long.
+enfant-f|La voiture va passer.
+papa|Tu poses les cubes, Nina ?
+enfant-f|Oui, papa.
+narrateur|Nina pose un cube trop vite.
+narrateur|Puis un autre, trop haut.
+enfant-f|Plus haut !
+narrateur|Le pont penche d'un coup, vers le sol.
+narrateur|Les cubes tombent près du tabouret.
+narrateur|Ça fait un bruit sec.
+enfant-f|Oh.
+narrateur|Nina reste surprise, les mains ouvertes.
 narrateur|Sa poitrine va trop vite.
-enfant-f|C'est trop. Je suis fâchée.
-papa|Le pont est tombé. Tu es fâchée.
-papa|On souffle.
-narrateur|Nina souffle.
-narrateur|Un grand souffle.
-papa|On fait une pause.
-narrateur|Nina s'assoit.
-narrateur|Elle pose les mains sur ses genoux.
-narrateur|Elle souffle encore.
-narrateur|La pause est calme.
-narrateur|Son ventre se desserre.
-narrateur|La pluie continue sur le toit.
-enfant-f|Je souffle. Je fais une pause.
-papa|Tu as soufflé. Tu as fait une pause.
-maman|Bravo, Nina. J'ai entendu. C'est calme.
-papa|Tu veux reprendre, tout doucement ?
-enfant-f|Oui. Un petit pont.
-narrateur|Nina reprend un cube.
-narrateur|Le pont est petit.
-narrateur|Il tient.</t>
+narrateur|Le sourire de Nina disparaît.
+enfant-f|C'est trop, papa.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois les cubes, Nina ?
+enfant-f|Oui, papa.
+maman|Tes mains sont chaudes, Nina ?
+enfant-f|Un peu, maman.
+narrateur|Un éclat de tabouret tremble, près du sol.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>pluie,cubes,soupe</t>
+          <t>voiture,cubes,soupe</t>
         </is>
       </c>
     </row>
@@ -1403,12 +1414,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Le pont tombe. Que fait Nina ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le pont tombe. Que fait &lt;emphasis level="moderate"&gt;Nina&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Le pont tombe. Que fait Ferdinand ?</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Le pont tombe. Que fait &lt;emphasis&gt;Nina&lt;/emphasis&gt; ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1471,18 +1482,18 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.24</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1497,34 +1508,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Nina</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1533,23 +1548,23 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=le_pont_tombe_que_fait_nina; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1582,17 +1597,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Nina a soufflé. Elle a fait une pause. Au salon, le petit pont tient. La voiture en bois peut attendre. Elle passera après. Plus tard, maman l'appelle. Nina, tu viens ? La soupe est prête. On range un cube, puis on y va. Dans la cuisine, une cuillère glisse. Ça fait un bruit fort dans le saladier. La vapeur de soupe est chaude. Nina sent encore son ventre. C'est trop. Je souffle. Je fais une pause. Oui. Tu t'assois près de moi. Nina s'assoit près de maman. La chaise ne bouge plus. Elle souffle. Elle fait une pause. Tu as soufflé. Tu as fait une pause. Puis tu reprends. Bravo. La soupe sent bon. Je suis plus calme.</t>
+          <t>Nina veut le pont, tout de suite. Je mets tout, maintenant ! Les cubes restent par terre, près du tabouret. Les mots se bousculent dans sa bouche. Trop vite. Nina avance les mains, trop vite. Puis elle s'arrête. Elle referme la bouche. Personne ne parle, un moment. Elle observe les cubes, un instant. Elle écoute le salon, près du bois. Pouh. Nina souffle une fois. Elle souffle une deuxième fois. Elle s'assoit près du tabouret. Elle fait une pause. Ses mains se posent sur ses genoux. La poitrine ralentit un peu. Tu restes un peu, Nina ? Oui, papa. Merci, Nina. Papa reste à la même hauteur. Le pain sent bon, depuis la cuisine. Il est tiède. Nina reprend un cube, sans se presser. Elle le pose sur un autre. Tu le vois, le cube ? Oui, papa. Il tient, Nina ? Oui, maman. Le pont a deux cubes, tout petits. Il tient ! Le pont est petit, Nina ? Oui, papa. Le ventre de Nina se desserre. Les épaules se relèvent un peu. La voiture attend à côté, sans rouler. Elle passera après. Nina, tu viens ? La soupe est prête. On y va, vers la cuisine ? Oui. Nina glisse la main sur le bois du tabouret. Le petit point.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Nina a soufflé. Elle a fait une pause. Au salon, le petit pont tient. La voiture en bois peut attendre. Elle passera après. Plus tard, maman l'appelle. Nina, tu viens ? La soupe est prête. On range un cube, puis on y va. Dans la cuisine, une cuillère glisse. Ça fait un bruit fort dans le saladier. La vapeur de soupe est chaude. Nina sent encore son ventre. C'est trop. Je souffle. Je fais une pause. Oui. Tu t'assois près de moi. Nina s'assoit près de maman. La chaise ne bouge plus. Elle souffle. Elle fait une pause. Tu as soufflé. Tu as fait une pause. Puis tu reprends. Bravo. La soupe sent bon. Je suis plus calme.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nina veut le pont, tout de suite. Je mets tout, maintenant ! Les cubes restent par terre, près du tabouret. Les mots se bousculent dans sa bouche. Trop vite. Nina avance les mains, trop vite. Puis elle s'arrête. Elle referme la bouche. Personne ne parle, un moment. Elle observe les cubes, un instant. Elle écoute le salon, près du bois. Pouh. Nina &lt;emphasis level="moderate"&gt;souffle&lt;/emphasis&gt; une fois. Elle souffle une deuxième fois. Elle s'assoit près du tabouret. Elle fait une pause. Ses mains se posent sur ses genoux. La poitrine ralentit un peu. Tu restes un peu, Nina ? Oui, papa. Merci, Nina. Papa reste à la même hauteur. Le pain sent bon, depuis la cuisine. Il est tiède. Nina reprend un cube, sans se presser. Elle le pose sur un autre. Tu le vois, le cube ? Oui, papa. Il tient, Nina ? Oui, maman. Le pont a deux cubes, tout petits. Il tient ! Le pont est petit, Nina ? Oui, papa. Le ventre de Nina se desserre. Les épaules se relèvent un peu. La voiture attend à côté, sans rouler. Elle passera après. Nina, tu viens ? La soupe est prête. On y va, vers la cuisine ? Oui. Nina glisse la main sur le bois du tabouret. Le petit point.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Ferdinand a soufflé. Il a fait une &lt;emphasis&gt;pause&lt;/emphasis&gt;. Au salon, puis à la cuisine. Papa et maman étaient là. [pause]</t>
+          <t>Nina veut le pont, tout de suite. Je mets tout, maintenant ! Les cubes restent par terre, près du tabouret. Les mots se bousculent dans sa bouche. Trop vite. Nina avance les mains, trop vite. Puis elle s'arrête. Elle referme la bouche. Personne ne parle, un moment. Elle observe les cubes, un instant. Elle écoute le salon, près du bois. Pouh. Nina &lt;emphasis&gt;souffle&lt;/emphasis&gt; une fois. Elle souffle une deuxième fois. Elle s'assoit près du tabouret. Elle fait une pause. Ses mains se posent sur ses genoux. La poitrine ralentit un peu. Tu restes un peu, Nina ? Oui, papa. Merci, Nina. Papa reste à la même hauteur. Le pain sent bon, depuis la cuisine. Il est tiède. Nina reprend un cube, sans se presser. Elle le pose sur un autre. Tu le vois, le cube ? Oui, papa. Il tient, Nina ? Oui, maman. Le pont a deux cubes, tout petits. Il tient ! Le pont est petit, Nina ? Oui, papa. Le ventre de Nina se desserre. Les épaules se relèvent un peu. La voiture attend à côté, sans rouler. Elle passera après. Nina, tu viens ? La soupe est prête. On y va, vers la cuisine ? Oui. Nina glisse la main sur le bois du tabouret. Le petit point. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1639,7 +1654,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1647,10 +1662,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.12</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1673,30 +1688,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>pause</t>
+          <t>souffle</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1705,10 +1720,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1721,37 +1736,60 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_souffle_elle_fait_une_pause; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Nina a soufflé.
-narrateur|Elle a fait une pause.
-narrateur|Au salon, le petit pont tient.
-papa|La voiture en bois peut attendre.
+          <t>narrateur|Nina veut le pont, tout de suite.
+enfant-f|Je mets tout, maintenant !
+narrateur|Les cubes restent par terre, près du tabouret.
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-f|Trop vite.
+narrateur|Nina avance les mains, trop vite.
+narrateur|Puis elle s'arrête.
+narrateur|Elle referme la bouche.
+narrateur|Personne ne parle, un moment.
+narrateur|Elle observe les cubes, un instant.
+narrateur|Elle écoute le salon, près du bois.
+enfant-f|Pouh.
+narrateur|Nina souffle une fois.
+narrateur|Elle souffle une deuxième fois.
+narrateur|Elle s'assoit près du tabouret.
+narrateur|Elle fait une pause.
+narrateur|Ses mains se posent sur ses genoux.
+narrateur|La poitrine ralentit un peu.
+papa|Tu restes un peu, Nina ?
+enfant-f|Oui, papa.
+papa|Merci, Nina.
+narrateur|Papa reste à la même hauteur.
+maman|Le pain sent bon, depuis la cuisine.
+enfant-f|Il est tiède.
+narrateur|Nina reprend un cube, sans se presser.
+narrateur|Elle le pose sur un autre.
+papa|Tu le vois, le cube ?
+enfant-f|Oui, papa.
+maman|Il tient, Nina ?
+enfant-f|Oui, maman.
+narrateur|Le pont a deux cubes, tout petits.
+enfant-f|Il tient !
+papa|Le pont est petit, Nina ?
+enfant-f|Oui, papa.
+narrateur|Le ventre de Nina se desserre.
+narrateur|Les épaules se relèvent un peu.
+narrateur|La voiture attend à côté, sans rouler.
 enfant-f|Elle passera après.
-narrateur|Plus tard, maman l'appelle.
-maman|Nina, tu viens ? La soupe est prête.
-papa|On range un cube, puis on y va.
-narrateur|Dans la cuisine, une cuillère glisse.
-narrateur|Ça fait un bruit fort dans le saladier.
-narrateur|La vapeur de soupe est chaude.
-narrateur|Nina sent encore son ventre.
-enfant-f|C'est trop. Je souffle. Je fais une pause.
-maman|Oui. Tu t'assois près de moi.
-narrateur|Nina s'assoit près de maman.
-narrateur|La chaise ne bouge plus.
-narrateur|Elle souffle.
-narrateur|Elle fait une pause.
-maman|Tu as soufflé. Tu as fait une pause.
-papa|Puis tu reprends. Bravo.
-enfant-f|La soupe sent bon. Je suis plus calme.</t>
+maman|Nina, tu viens ?
+maman|La soupe est prête.
+papa|On y va, vers la cuisine ?
+enfant-f|Oui.
+narrateur|Nina glisse la main sur le bois du tabouret.
+enfant-f|Le petit point.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>cuisine,cuillere</t>
+          <t>cubes</t>
         </is>
       </c>
     </row>
@@ -1778,17 +1816,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nina pose un cube sur le bord. Le pont, au salon, est petit. Il tient, papa. Oui. Tu as fini de ranger ce cube ? Oui. La soupe attend. Tu t'assois ? Nina s'assoit à table. Le pain est encore chaud. La pluie fait encore des petits coups.</t>
+          <t>Ils passent vers la cuisine. La vapeur de soupe est chaude. Ça sent fort, maman. Tu la sens, la vapeur ? Oui, maman. Le tabouret reste à la porte, vers le salon. Une casserole glisse vers le bord. Ça fait un bruit fort, près du feu. Elle glisse ! Nina avance trop vite, les mains ouvertes. Sa poitrine repart trop vite. Oh. Nina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la casserole, un instant. Elle écoute la cuisine, près du feu. Sur le bois, un éclat de tabouret luit. Là, sur le bois. Nina souffle une fois. Elle attend, assise un moment. Pouh. On tient le bord ? Oui, papa. Papa pousse la casserole, sans se presser. La soupe reste dans le fond, Nina ? Oui, maman. Nina fait une pause, les mains sur les genoux. Tu restes près de nous, Nina ? Oui, papa. La vapeur monte, plus lente. Elle est chaude. Tes mains sont au chaud, Nina ? Un peu, maman. La casserole est calme, Nina ? Oui, papa. Un rayon passe sur le bois du tabouret. Il allume le bois. Le tabouret tient à la porte, vers le salon. Le pont est là-bas.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Nina pose un cube sur le bord. Le pont, au salon, est petit. Il tient, papa. Oui. Tu as fini de ranger ce cube ? Oui. La soupe attend. Tu t'assois ? Nina s'assoit à table. Le pain est encore chaud. La pluie fait encore des petits coups.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ils passent vers la cuisine. La vapeur de soupe est chaude. Ça sent fort, maman. Tu la sens, la vapeur ? Oui, maman. Le tabouret reste à la porte, vers le salon. Une casserole glisse vers le bord. Ça fait un bruit fort, près du feu. Elle glisse ! Nina avance trop vite, les mains ouvertes. Sa poitrine repart trop vite. Oh. Nina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la casserole, un instant. Elle écoute la cuisine, près du feu. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de tabouret&lt;/emphasis&gt; luit. Là, sur le bois. Nina souffle une fois. Elle attend, assise un moment. Pouh. On tient le bord ? Oui, papa. Papa pousse la casserole, sans se presser. La soupe reste dans le fond, Nina ? Oui, maman. Nina fait une pause, les mains sur les genoux. Tu restes près de nous, Nina ? Oui, papa. La vapeur monte, plus lente. Elle est chaude. Tes mains sont au chaud, Nina ? Un peu, maman. La casserole est calme, Nina ? Oui, papa. Un rayon passe sur le bois du tabouret. Il allume le bois. Le tabouret tient à la porte, vers le salon. Le pont est là-bas.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Ferdinand pose un cube. Le pont est petit. [pause]</t>
+          <t>Ils passent vers la cuisine. La vapeur de soupe est chaude. Ça sent fort, maman. Tu la sens, la vapeur ? Oui, maman. Le tabouret reste à la porte, vers le salon. Une casserole glisse vers le bord. Ça fait un bruit fort, près du feu. Elle glisse ! Nina avance trop vite, les mains ouvertes. Sa poitrine repart trop vite. Oh. Nina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe la casserole, un instant. Elle écoute la cuisine, près du feu. Sur le bois, un &lt;emphasis&gt;éclat de tabouret&lt;/emphasis&gt; luit. Là, sur le bois. Nina souffle une fois. Elle attend, assise un moment. Pouh. On tient le bord ? Oui, papa. Papa pousse la casserole, sans se presser. La soupe reste dans le fond, Nina ? Oui, maman. Nina fait une pause, les mains sur les genoux. Tu restes près de nous, Nina ? Oui, papa. La vapeur monte, plus lente. Elle est chaude. Tes mains sont au chaud, Nina ? Un peu, maman. La casserole est calme, Nina ? Oui, papa. Un rayon passe sur le bois du tabouret. Il allume le bois. Le tabouret tient à la porte, vers le salon. Le pont est là-bas. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1835,7 +1873,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1843,10 +1881,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.12</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1867,28 +1905,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de tabouret</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1897,10 +1939,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.96</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1911,23 +1953,58 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=casserole_glisse_corps_repart_elle_s_arrete; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Nina pose un cube sur le bord.
-narrateur|Le pont, au salon, est petit.
-enfant-f|Il tient, papa.
-papa|Oui. Tu as fini de ranger ce cube ?
-enfant-f|Oui.
-maman|La soupe attend. Tu t'assois ?
-narrateur|Nina s'assoit à table.
-narrateur|Le pain est encore chaud.
-narrateur|La pluie fait encore des petits coups.</t>
+          <t>narrateur|Ils passent vers la cuisine.
+narrateur|La vapeur de soupe est chaude.
+enfant-f|Ça sent fort, maman.
+maman|Tu la sens, la vapeur ?
+enfant-f|Oui, maman.
+narrateur|Le tabouret reste à la porte, vers le salon.
+narrateur|Une casserole glisse vers le bord.
+narrateur|Ça fait un bruit fort, près du feu.
+enfant-f|Elle glisse !
+narrateur|Nina avance trop vite, les mains ouvertes.
+narrateur|Sa poitrine repart trop vite.
+enfant-f|Oh.
+narrateur|Nina refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe la casserole, un instant.
+narrateur|Elle écoute la cuisine, près du feu.
+narrateur|Sur le bois, un éclat de tabouret luit.
+enfant-f|Là, sur le bois.
+narrateur|Nina souffle une fois.
+narrateur|Elle attend, assise un moment.
+enfant-f|Pouh.
+papa|On tient le bord ?
+enfant-f|Oui, papa.
+narrateur|Papa pousse la casserole, sans se presser.
+maman|La soupe reste dans le fond, Nina ?
+enfant-f|Oui, maman.
+narrateur|Nina fait une pause, les mains sur les genoux.
+papa|Tu restes près de nous, Nina ?
+enfant-f|Oui, papa.
+narrateur|La vapeur monte, plus lente.
+enfant-f|Elle est chaude.
+maman|Tes mains sont au chaud, Nina ?
+enfant-f|Un peu, maman.
+papa|La casserole est calme, Nina ?
+enfant-f|Oui, papa.
+maman|Un rayon passe sur le bois du tabouret.
+enfant-f|Il allume le bois.
+narrateur|Le tabouret tient à la porte, vers le salon.
+enfant-f|Le pont est là-bas.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>soupe</t>
+          <t>cuisine,casserole</t>
         </is>
       </c>
     </row>
@@ -1954,17 +2031,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai soufflé. J'ai fait une pause. Bravo, Nina. Le pont est petit. La soupe est là.</t>
+          <t>Ils restent près de la soupe. Tu t'assois, Nina ? Oui, maman. Nina s'assoit près du tabouret. Le petit pont, au salon, est petit ? Il tient, papa. Le petit pont a failli rester en tas. Il a une trace de bois. Tu la vois, la trace ? Oui, maman. La soupe est là, Nina. Elle sent bon. Le pain est tiède, sous les doigts. Et la soupe, maman. Oui, dans l'air. La cuisine est calme, Nina ? Oui, papa. Un éclat de tabouret tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai soufflé. J'ai fait une pause. Bravo, Nina. Le pont est petit. La soupe est là.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la soupe. Tu t'assois, Nina ? Oui, maman. Nina s'assoit près du tabouret. Le petit pont, au salon, est petit ? Il tient, papa. Le petit pont a failli rester en tas. Il a une trace de bois. Tu la vois, la trace ? Oui, maman. La soupe est là, Nina. Elle sent bon. Le pain est tiède, sous les doigts. Et la soupe, maman. Oui, dans l'air. La cuisine est calme, Nina ? Oui, papa. Un &lt;emphasis level="moderate"&gt;éclat de tabouret&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;L'histoire est finie.&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la soupe. Tu t'assois, Nina ? Oui, maman. Nina s'assoit près du tabouret. Le petit pont, au salon, est petit ? Il tient, papa. Le petit pont a failli rester en tas. Il a une trace de bois. Tu la vois, la trace ? Oui, maman. La soupe est là, Nina. Elle sent bon. Le pain est tiède, sous les doigts. Et la soupe, maman. Oui, dans l'air. La cuisine est calme, Nina ? Oui, papa. Un &lt;emphasis&gt;éclat de tabouret&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2011,18 +2088,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.2</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2031,12 +2108,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2045,17 +2122,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de tabouret</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2064,11 +2145,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2077,26 +2158,50 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai soufflé. J'ai fait une pause.
-maman|Bravo, Nina.
-papa|Le pont est petit. La soupe est là.</t>
+          <t>narrateur|Ils restent près de la soupe.
+maman|Tu t'assois, Nina ?
+enfant-f|Oui, maman.
+narrateur|Nina s'assoit près du tabouret.
+papa|Le petit pont, au salon, est petit ?
+enfant-f|Il tient, papa.
+narrateur|Le petit pont a failli rester en tas.
+enfant-f|Il a une trace de bois.
+maman|Tu la vois, la trace ?
+enfant-f|Oui, maman.
+papa|La soupe est là, Nina.
+enfant-f|Elle sent bon.
+narrateur|Le pain est tiède, sous les doigts.
+enfant-f|Et la soupe, maman.
+maman|Oui, dans l'air.
+papa|La cuisine est calme, Nina ?
+enfant-f|Oui, papa.
+narrateur|Un éclat de tabouret tient sur le bois.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>soupe</t>
         </is>
       </c>
     </row>
@@ -2117,7 +2222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2181,6 +2286,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>